<commit_message>
feat(combat): G07-P1-B4 execute effect lifecycle
</commit_message>
<xml_diff>
--- a/config/data/StateSlotReset.xlsx
+++ b/config/data/StateSlotReset.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -584,6 +584,19 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="B9" t="n">
+        <v>24003</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>BattleStart</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>